<commit_message>
auto(MT): 3h refresh 2026-05-17T05:06Z
</commit_message>
<xml_diff>
--- a/summary_2026-05-17.xlsx
+++ b/summary_2026-05-17.xlsx
@@ -53001,10 +53001,10 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="C4" s="11" t="n">
-        <v>714</v>
+        <v>727</v>
       </c>
       <c r="D4" s="11" t="n">
         <v>63</v>
@@ -53076,10 +53076,10 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1336</v>
+        <v>1349</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>125</v>
@@ -53105,7 +53105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I85"/>
+  <dimension ref="A1:I72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -53562,7 +53562,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Vania Agius Tabone</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -53573,12 +53573,12 @@
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Vania Agius Tabone</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1839054247500559</t>
+          <t>1321288733281834</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -53597,23 +53597,23 @@
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>Vania Agius Tabone</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr"/>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Vania Agius Tabone</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>1321288733281834</t>
+          <t>2380595315785369</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -53648,7 +53648,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2380595315785369</t>
+          <t>1683215979770872</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -53683,7 +53683,7 @@
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>1683215979770872</t>
+          <t>1644456073494625</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -53702,7 +53702,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Luke Said</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -53713,12 +53713,12 @@
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Luke Said</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1644456073494625</t>
+          <t>1513928240522335</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -53737,23 +53737,23 @@
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>Luke Said</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr"/>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Luke Said</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>1513928240522335</t>
+          <t>3871030129694577</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -53788,7 +53788,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>3871030129694577</t>
+          <t>945783808284948</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -53807,23 +53807,23 @@
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Alex Borg</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr"/>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>945783808284948</t>
+          <t>958905883437296</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -53833,7 +53833,7 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr"/>
@@ -53842,7 +53842,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Alex Borg</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -53853,12 +53853,12 @@
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>958905883437296</t>
+          <t>1488053072699926</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -53877,7 +53877,7 @@
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
@@ -53888,12 +53888,12 @@
       <c r="C24" s="11" t="inlineStr"/>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>1488053072699926</t>
+          <t>2026943771563450</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -53928,7 +53928,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026943771563450</t>
+          <t>1003888061994637</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
@@ -53947,7 +53947,7 @@
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
@@ -53958,12 +53958,12 @@
       <c r="C26" s="11" t="inlineStr"/>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>1003888061994637</t>
+          <t>2146428012843469</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -53982,7 +53982,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>George Vital Zammit</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -53993,12 +53993,12 @@
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t xml:space="preserve">George Vital Zammit Kandidat PN </t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2146428012843469</t>
+          <t>864621386654273</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
@@ -54017,7 +54017,7 @@
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>George Vital Zammit</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
@@ -54028,12 +54028,12 @@
       <c r="C28" s="11" t="inlineStr"/>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">George Vital Zammit Kandidat PN </t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>864621386654273</t>
+          <t>2423292861498917</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
@@ -54068,7 +54068,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2423292861498917</t>
+          <t>1690336838632544</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
@@ -54087,7 +54087,7 @@
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Frank Anthony Tabone</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
@@ -54098,12 +54098,12 @@
       <c r="C30" s="11" t="inlineStr"/>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Frank Anthony Tabone</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>1690336838632544</t>
+          <t>1545046643935454</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
@@ -54122,23 +54122,23 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Frank Anthony Tabone</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Frank Anthony Tabone</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1545046643935454</t>
+          <t>1398617112285911</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
@@ -54173,7 +54173,7 @@
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>1398617112285911</t>
+          <t>1501901271598336</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
@@ -54192,7 +54192,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -54203,12 +54203,12 @@
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1501901271598336</t>
+          <t>1862149954473065</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
@@ -54227,7 +54227,7 @@
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Carlos Zarb</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
@@ -54238,12 +54238,12 @@
       <c r="C34" s="11" t="inlineStr"/>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Carlos Zarb</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>1862149954473065</t>
+          <t>939653538880289</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
@@ -54262,23 +54262,23 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Carlos Zarb</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Carlos Zarb</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>939653538880289</t>
+          <t>1463878141656116</t>
         </is>
       </c>
       <c r="F35" s="8" t="inlineStr">
@@ -54288,7 +54288,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
@@ -54297,7 +54297,7 @@
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Rachel Williams</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
@@ -54308,12 +54308,12 @@
       <c r="C36" s="11" t="inlineStr"/>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Williams Hymie Rubetta</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>1463878141656116</t>
+          <t>1534731544699810</t>
         </is>
       </c>
       <c r="F36" s="8" t="inlineStr">
@@ -54332,23 +54332,23 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Rachel Williams</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Williams Hymie Rubetta</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1534731544699810</t>
+          <t>1531533181939436</t>
         </is>
       </c>
       <c r="F37" s="8" t="inlineStr">
@@ -54367,7 +54367,7 @@
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
@@ -54378,12 +54378,12 @@
       <c r="C38" s="11" t="inlineStr"/>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>1531533181939436</t>
+          <t>1246323254060158</t>
         </is>
       </c>
       <c r="F38" s="8" t="inlineStr">
@@ -54402,23 +54402,23 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Julian Borg</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Julian Borg</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1246323254060158</t>
+          <t>26732437223117722</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
@@ -54437,23 +54437,23 @@
     <row r="40">
       <c r="A40" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Paula Mifsud Bonnici</t>
         </is>
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr"/>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Maria Mifsud Bonnici</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
         <is>
-          <t>26632426153093650</t>
+          <t>2435722906905478</t>
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr">
@@ -54472,7 +54472,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Julian Borg</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -54483,12 +54483,12 @@
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Julian Borg</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>26732437223117722</t>
+          <t>978460398253114</t>
         </is>
       </c>
       <c r="F41" s="8" t="inlineStr">
@@ -54507,23 +54507,23 @@
     <row r="42">
       <c r="A42" s="11" t="inlineStr">
         <is>
-          <t>Paula Mifsud Bonnici</t>
+          <t>Robert Abela</t>
         </is>
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr"/>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Maria Mifsud Bonnici</t>
+          <t>Anthony Agius Decelis</t>
         </is>
       </c>
       <c r="E42" s="11" t="inlineStr">
         <is>
-          <t>2435722906905478</t>
+          <t>2064151104521171</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
@@ -54542,23 +54542,23 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Jesmond Bonello</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Bonello Jesmond</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>978460398253114</t>
+          <t>26918648411088542</t>
         </is>
       </c>
       <c r="F43" s="8" t="inlineStr">
@@ -54577,7 +54577,7 @@
     <row r="44">
       <c r="A44" s="11" t="inlineStr">
         <is>
-          <t>Robert Abela</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B44" s="11" t="inlineStr">
@@ -54588,12 +54588,12 @@
       <c r="C44" s="11" t="inlineStr"/>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Anthony Agius Decelis</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E44" s="11" t="inlineStr">
         <is>
-          <t>2064151104521171</t>
+          <t>1504143931434748</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
@@ -54612,7 +54612,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Jesmond Bonello</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -54623,12 +54623,12 @@
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Bonello Jesmond</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>26918648411088542</t>
+          <t>1518066693268355</t>
         </is>
       </c>
       <c r="F45" s="8" t="inlineStr">
@@ -54647,7 +54647,7 @@
     <row r="46">
       <c r="A46" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B46" s="11" t="inlineStr">
@@ -54658,12 +54658,12 @@
       <c r="C46" s="11" t="inlineStr"/>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
         <is>
-          <t>1504143931434748</t>
+          <t>1985551062067193</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
@@ -54673,7 +54673,7 @@
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr"/>
@@ -54682,7 +54682,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Tania Borg</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -54693,12 +54693,12 @@
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Tania Borg For District 9 &amp; 10</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>1518066693268355</t>
+          <t>974302048675707</t>
         </is>
       </c>
       <c r="F47" s="8" t="inlineStr">
@@ -54708,7 +54708,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="H47" t="inlineStr"/>
@@ -54717,7 +54717,7 @@
     <row r="48">
       <c r="A48" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Tania Borg</t>
         </is>
       </c>
       <c r="B48" s="11" t="inlineStr">
@@ -54728,12 +54728,12 @@
       <c r="C48" s="11" t="inlineStr"/>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Tania Borg For District 9 &amp; 10</t>
         </is>
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
-          <t>1985551062067193</t>
+          <t>1025067929953806</t>
         </is>
       </c>
       <c r="F48" s="8" t="inlineStr">
@@ -54752,7 +54752,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Tania Borg</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -54763,12 +54763,12 @@
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Tania Borg For District 9 &amp; 10</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>974302048675707</t>
+          <t>962084660082350</t>
         </is>
       </c>
       <c r="F49" s="8" t="inlineStr">
@@ -54787,7 +54787,7 @@
     <row r="50">
       <c r="A50" s="11" t="inlineStr">
         <is>
-          <t>Tania Borg</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="B50" s="11" t="inlineStr">
@@ -54798,12 +54798,12 @@
       <c r="C50" s="11" t="inlineStr"/>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Tania Borg For District 9 &amp; 10</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>1025067929953806</t>
+          <t>1430222058857743</t>
         </is>
       </c>
       <c r="F50" s="8" t="inlineStr">
@@ -54822,23 +54822,23 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>John Baptist Camilleri</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>John Baptist Camilleri</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>962084660082350</t>
+          <t>993445096523240</t>
         </is>
       </c>
       <c r="F51" s="8" t="inlineStr">
@@ -54848,7 +54848,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
@@ -54857,23 +54857,23 @@
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Julian Borg</t>
         </is>
       </c>
       <c r="B52" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr"/>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Julian Borg</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
         <is>
-          <t>1430222058857743</t>
+          <t>1006210008553971</t>
         </is>
       </c>
       <c r="F52" s="8" t="inlineStr">
@@ -54883,7 +54883,7 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr"/>
@@ -54892,23 +54892,23 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>916777084726084</t>
+          <t>2068362770561777</t>
         </is>
       </c>
       <c r="F53" s="8" t="inlineStr">
@@ -54918,7 +54918,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H53" t="inlineStr"/>
@@ -54927,23 +54927,23 @@
     <row r="54">
       <c r="A54" s="11" t="inlineStr">
         <is>
-          <t>John Baptist Camilleri</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B54" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr"/>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>John Baptist Camilleri</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
-          <t>993445096523240</t>
+          <t>996986282983288</t>
         </is>
       </c>
       <c r="F54" s="8" t="inlineStr">
@@ -54962,23 +54962,23 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Julian Borg</t>
+          <t>Cressida Galea</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Julian Borg</t>
+          <t>Cressida Galea - Ekonomista</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>1006210008553971</t>
+          <t>4353539594976013</t>
         </is>
       </c>
       <c r="F55" s="8" t="inlineStr">
@@ -54997,23 +54997,23 @@
     <row r="56">
       <c r="A56" s="11" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Cressida Galea</t>
         </is>
       </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr"/>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Cressida Galea - Ekonomista</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>2068362770561777</t>
+          <t>1656439582071818</t>
         </is>
       </c>
       <c r="F56" s="8" t="inlineStr">
@@ -55032,7 +55032,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Kaydem Schembri</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -55043,12 +55043,12 @@
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Kaydem Schembri</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>996986282983288</t>
+          <t>996190969523573</t>
         </is>
       </c>
       <c r="F57" s="8" t="inlineStr">
@@ -55067,23 +55067,23 @@
     <row r="58">
       <c r="A58" s="11" t="inlineStr">
         <is>
-          <t>Cressida Galea</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr"/>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Cressida Galea - Ekonomista</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="E58" s="11" t="inlineStr">
         <is>
-          <t>4353539594976013</t>
+          <t>1625614571830540</t>
         </is>
       </c>
       <c r="F58" s="8" t="inlineStr">
@@ -55102,23 +55102,23 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Cressida Galea</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Cressida Galea - Ekonomista</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>1656439582071818</t>
+          <t>3276604689166967</t>
         </is>
       </c>
       <c r="F59" s="8" t="inlineStr">
@@ -55128,7 +55128,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H59" t="inlineStr"/>
@@ -55137,7 +55137,7 @@
     <row r="60">
       <c r="A60" s="11" t="inlineStr">
         <is>
-          <t>Kaydem Schembri</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B60" s="11" t="inlineStr">
@@ -55148,12 +55148,12 @@
       <c r="C60" s="11" t="inlineStr"/>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>Kaydem Schembri</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E60" s="11" t="inlineStr">
         <is>
-          <t>996190969523573</t>
+          <t>2115618699296224</t>
         </is>
       </c>
       <c r="F60" s="8" t="inlineStr">
@@ -55163,7 +55163,7 @@
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr"/>
@@ -55172,23 +55172,23 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Momentum</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>1625614571830540</t>
+          <t>949145677752982</t>
         </is>
       </c>
       <c r="F61" s="8" t="inlineStr">
@@ -55198,7 +55198,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H61" t="inlineStr"/>
@@ -55207,23 +55207,23 @@
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr"/>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr">
         <is>
-          <t>3984183268548920</t>
+          <t>1470892497314849</t>
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
@@ -55233,7 +55233,7 @@
       </c>
       <c r="G62" s="11" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H62" s="11" t="inlineStr"/>
@@ -55242,23 +55242,23 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>3276604689166967</t>
+          <t>1997023797841290</t>
         </is>
       </c>
       <c r="F63" s="8" t="inlineStr">
@@ -55277,7 +55277,7 @@
     <row r="64">
       <c r="A64" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Lorna Borg Vassallo</t>
         </is>
       </c>
       <c r="B64" s="11" t="inlineStr">
@@ -55288,12 +55288,12 @@
       <c r="C64" s="11" t="inlineStr"/>
       <c r="D64" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Lorna Borġ Vassallo</t>
         </is>
       </c>
       <c r="E64" s="11" t="inlineStr">
         <is>
-          <t>2115618699296224</t>
+          <t>982543764707676</t>
         </is>
       </c>
       <c r="F64" s="8" t="inlineStr">
@@ -55312,23 +55312,23 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>John Baptist Camilleri</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>John Baptist Camilleri</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>949145677752982</t>
+          <t>35349534414693500</t>
         </is>
       </c>
       <c r="F65" s="8" t="inlineStr">
@@ -55338,7 +55338,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H65" t="inlineStr"/>
@@ -55347,23 +55347,23 @@
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Katya De Giovanni</t>
         </is>
       </c>
       <c r="B66" s="11" t="inlineStr">
         <is>
-          <t>Momentum</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C66" s="11" t="inlineStr"/>
       <c r="D66" s="11" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Katya De Giovanni</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
         <is>
-          <t>1470892497314849</t>
+          <t>26625959597085054</t>
         </is>
       </c>
       <c r="F66" s="8" t="inlineStr">
@@ -55373,7 +55373,7 @@
       </c>
       <c r="G66" s="11" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="H66" s="11" t="inlineStr"/>
@@ -55382,23 +55382,23 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Momentum</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>1997023797841290</t>
+          <t>909198525476235</t>
         </is>
       </c>
       <c r="F67" s="8" t="inlineStr">
@@ -55408,7 +55408,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="H67" t="inlineStr"/>
@@ -55417,7 +55417,7 @@
     <row r="68">
       <c r="A68" s="11" t="inlineStr">
         <is>
-          <t>Lorna Borg Vassallo</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B68" s="11" t="inlineStr">
@@ -55428,12 +55428,12 @@
       <c r="C68" s="11" t="inlineStr"/>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>Lorna Borġ Vassallo</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
         <is>
-          <t>982543764707676</t>
+          <t>2050566099220285</t>
         </is>
       </c>
       <c r="F68" s="8" t="inlineStr">
@@ -55443,7 +55443,7 @@
       </c>
       <c r="G68" s="11" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="H68" s="11" t="inlineStr"/>
@@ -55452,7 +55452,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>John Baptist Camilleri</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -55463,12 +55463,12 @@
       <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
-          <t>John Baptist Camilleri</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>35349534414693500</t>
+          <t>1677247313280464</t>
         </is>
       </c>
       <c r="F69" s="8" t="inlineStr">
@@ -55478,7 +55478,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="H69" t="inlineStr"/>
@@ -55487,7 +55487,7 @@
     <row r="70">
       <c r="A70" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Nigel Vella</t>
         </is>
       </c>
       <c r="B70" s="11" t="inlineStr">
@@ -55498,12 +55498,12 @@
       <c r="C70" s="11" t="inlineStr"/>
       <c r="D70" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Nigel Vella</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
         <is>
-          <t>2489452081571575</t>
+          <t>1478044677100859</t>
         </is>
       </c>
       <c r="F70" s="8" t="inlineStr">
@@ -55513,7 +55513,7 @@
       </c>
       <c r="G70" s="11" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="H70" s="11" t="inlineStr"/>
@@ -55522,7 +55522,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Katya De Giovanni</t>
+          <t>Lorna Borg Vassallo</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -55533,12 +55533,12 @@
       <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Katya De Giovanni</t>
+          <t>Lorna Borġ Vassallo</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>26625959597085054</t>
+          <t>942778361908557</t>
         </is>
       </c>
       <c r="F71" s="8" t="inlineStr">
@@ -55548,7 +55548,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="H71" t="inlineStr"/>
@@ -55557,7 +55557,7 @@
     <row r="72">
       <c r="A72" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Lorna Borg Vassallo</t>
         </is>
       </c>
       <c r="B72" s="11" t="inlineStr">
@@ -55568,12 +55568,12 @@
       <c r="C72" s="11" t="inlineStr"/>
       <c r="D72" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Lorna Borġ Vassallo</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
         <is>
-          <t>1269656098669646</t>
+          <t>984647040762034</t>
         </is>
       </c>
       <c r="F72" s="8" t="inlineStr">
@@ -55583,466 +55583,11 @@
       </c>
       <c r="G72" s="11" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="H72" s="11" t="inlineStr"/>
       <c r="I72" s="11" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>Michael Piccinino</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>PN</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr"/>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>Michael Piccinino</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>909198525476235</t>
-        </is>
-      </c>
-      <c r="F73" s="8" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="11" t="inlineStr">
-        <is>
-          <t>Edward Cassar Delia</t>
-        </is>
-      </c>
-      <c r="B74" s="11" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
-      <c r="C74" s="11" t="inlineStr"/>
-      <c r="D74" s="11" t="inlineStr">
-        <is>
-          <t>Edward Cassar Delia</t>
-        </is>
-      </c>
-      <c r="E74" s="11" t="inlineStr">
-        <is>
-          <t>2050566099220285</t>
-        </is>
-      </c>
-      <c r="F74" s="8" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="G74" s="11" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="H74" s="11" t="inlineStr"/>
-      <c r="I74" s="11" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr"/>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>1751227829173959</t>
-        </is>
-      </c>
-      <c r="F75" s="8" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="11" t="inlineStr">
-        <is>
-          <t>Michael Piccinino</t>
-        </is>
-      </c>
-      <c r="B76" s="11" t="inlineStr">
-        <is>
-          <t>PN</t>
-        </is>
-      </c>
-      <c r="C76" s="11" t="inlineStr"/>
-      <c r="D76" s="11" t="inlineStr">
-        <is>
-          <t>Michael Piccinino</t>
-        </is>
-      </c>
-      <c r="E76" s="11" t="inlineStr">
-        <is>
-          <t>1677247313280464</t>
-        </is>
-      </c>
-      <c r="F76" s="8" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="G76" s="11" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="H76" s="11" t="inlineStr"/>
-      <c r="I76" s="11" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>Nigel Vella</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr"/>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>Nigel Vella</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>1478044677100859</t>
-        </is>
-      </c>
-      <c r="F77" s="8" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="11" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="B78" s="11" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
-      <c r="C78" s="11" t="inlineStr"/>
-      <c r="D78" s="11" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="E78" s="11" t="inlineStr">
-        <is>
-          <t>25743656911977946</t>
-        </is>
-      </c>
-      <c r="F78" s="8" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="G78" s="11" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="H78" s="11" t="inlineStr"/>
-      <c r="I78" s="11" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>Lorna Borg Vassallo</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr"/>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>Lorna Borġ Vassallo</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>942778361908557</t>
-        </is>
-      </c>
-      <c r="F79" s="8" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>2026-05-03</t>
-        </is>
-      </c>
-      <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="11" t="inlineStr">
-        <is>
-          <t>Lorna Borg Vassallo</t>
-        </is>
-      </c>
-      <c r="B80" s="11" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
-      <c r="C80" s="11" t="inlineStr"/>
-      <c r="D80" s="11" t="inlineStr">
-        <is>
-          <t>Lorna Borġ Vassallo</t>
-        </is>
-      </c>
-      <c r="E80" s="11" t="inlineStr">
-        <is>
-          <t>984647040762034</t>
-        </is>
-      </c>
-      <c r="F80" s="8" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="G80" s="11" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="H80" s="11" t="inlineStr"/>
-      <c r="I80" s="11" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr"/>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>4138793939597915</t>
-        </is>
-      </c>
-      <c r="F81" s="8" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr"/>
-      <c r="I81" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="11" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="B82" s="11" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
-      <c r="C82" s="11" t="inlineStr"/>
-      <c r="D82" s="11" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="E82" s="11" t="inlineStr">
-        <is>
-          <t>992931903251467</t>
-        </is>
-      </c>
-      <c r="F82" s="8" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="G82" s="11" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-      <c r="H82" s="11" t="inlineStr"/>
-      <c r="I82" s="11" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr"/>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>826788747138897</t>
-        </is>
-      </c>
-      <c r="F83" s="8" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>2026-04-26</t>
-        </is>
-      </c>
-      <c r="H83" t="inlineStr"/>
-      <c r="I83" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="11" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="B84" s="11" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
-      <c r="C84" s="11" t="inlineStr"/>
-      <c r="D84" s="11" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="E84" s="11" t="inlineStr">
-        <is>
-          <t>866748536435658</t>
-        </is>
-      </c>
-      <c r="F84" s="8" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="G84" s="11" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="H84" s="11" t="inlineStr"/>
-      <c r="I84" s="11" t="inlineStr"/>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr"/>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>937586149178445</t>
-        </is>
-      </c>
-      <c r="F85" s="8" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>2026-04-23</t>
-        </is>
-      </c>
-      <c r="H85" t="inlineStr"/>
-      <c r="I85" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -56115,19 +55660,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F79" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F80" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F81" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F82" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F83" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F84" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F85" r:id="rId82"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto(MT): 3h refresh 2026-05-17T09:06Z
</commit_message>
<xml_diff>
--- a/summary_2026-05-17.xlsx
+++ b/summary_2026-05-17.xlsx
@@ -53001,16 +53001,16 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="C4" s="11" t="n">
-        <v>727</v>
+        <v>730</v>
       </c>
       <c r="D4" s="11" t="n">
         <v>63</v>
       </c>
       <c r="E4" s="11" t="n">
-        <v>824</v>
+        <v>841</v>
       </c>
       <c r="F4" s="11" t="n">
         <v>177987</v>
@@ -53026,10 +53026,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C5" t="n">
-        <v>580</v>
+        <v>586</v>
       </c>
       <c r="D5" t="n">
         <v>58</v>
@@ -53076,16 +53076,16 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1349</v>
+        <v>1358</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>125</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>1543</v>
+        <v>1560</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>313057</v>
@@ -53105,7 +53105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I72"/>
+  <dimension ref="A1:I80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -53317,23 +53317,23 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr"/>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>1752525089454709</t>
+          <t>958788750313712</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -53352,7 +53352,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -53363,12 +53363,12 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>958788750313712</t>
+          <t>1732358601287330</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -53387,23 +53387,23 @@
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>David Caruana</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr"/>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>David Caruana</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>856712360814977</t>
+          <t>35705903765720926</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -53413,7 +53413,7 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr"/>
@@ -53422,23 +53422,23 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>4401025156884497</t>
+          <t>2516403832112892</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -53448,7 +53448,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -53457,7 +53457,7 @@
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
@@ -53468,12 +53468,12 @@
       <c r="C12" s="11" t="inlineStr"/>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>1680974129907056</t>
+          <t>1586602910140140</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -53483,7 +53483,7 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr"/>
@@ -53492,23 +53492,23 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1479722413058169</t>
+          <t>856712360814977</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -53527,7 +53527,7 @@
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
@@ -53538,12 +53538,12 @@
       <c r="C14" s="11" t="inlineStr"/>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>1426917766136513</t>
+          <t>1680974129907056</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -53562,7 +53562,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Vania Agius Tabone</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -53573,12 +53573,12 @@
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Vania Agius Tabone</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1321288733281834</t>
+          <t>1479722413058169</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -53597,23 +53597,23 @@
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr"/>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>2380595315785369</t>
+          <t>1426917766136513</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -53632,23 +53632,23 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Vania Agius Tabone</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Vania Agius Tabone</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1683215979770872</t>
+          <t>1321288733281834</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -53683,7 +53683,7 @@
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>1644456073494625</t>
+          <t>2380595315785369</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -53702,7 +53702,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Luke Said</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -53713,12 +53713,12 @@
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Luke Said</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1513928240522335</t>
+          <t>1683215979770872</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -53807,23 +53807,23 @@
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>Alex Borg</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr"/>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>958905883437296</t>
+          <t>1350786307104546</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -53833,7 +53833,7 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr"/>
@@ -53842,23 +53842,23 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1488053072699926</t>
+          <t>873330299113401</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -53868,7 +53868,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
@@ -53877,23 +53877,23 @@
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr"/>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>2026943771563450</t>
+          <t>1294864578834169</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -53903,7 +53903,7 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr"/>
@@ -53912,23 +53912,23 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Miriam Dalli</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Malta ESG Alliance</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1003888061994637</t>
+          <t>2377088586134238</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
@@ -53938,7 +53938,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -53947,23 +53947,23 @@
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Samantha Pace Gasan</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr"/>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Samantha Pace Gasan</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>2146428012843469</t>
+          <t>983555364558689</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -53973,7 +53973,7 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr"/>
@@ -53982,23 +53982,23 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>George Vital Zammit</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">George Vital Zammit Kandidat PN </t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>864621386654273</t>
+          <t>1272070931325786</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
@@ -54008,7 +54008,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
@@ -54017,23 +54017,23 @@
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr"/>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>2423292861498917</t>
+          <t>2431998763969509</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
@@ -54043,7 +54043,7 @@
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr"/>
@@ -54052,23 +54052,23 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>James Grech</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>James Grech</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1690336838632544</t>
+          <t>971268672293806</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
@@ -54078,7 +54078,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -54087,23 +54087,23 @@
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>Frank Anthony Tabone</t>
+          <t>James Grech</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr"/>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Frank Anthony Tabone</t>
+          <t>James Grech</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>1545046643935454</t>
+          <t>991693409986643</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
@@ -54113,7 +54113,7 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr"/>
@@ -54122,7 +54122,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>James Grech</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -54133,12 +54133,12 @@
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>James Grech</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1398617112285911</t>
+          <t>2662232900814818</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
@@ -54148,7 +54148,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
@@ -54157,23 +54157,23 @@
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Alex Borg</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr"/>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>1501901271598336</t>
+          <t>958905883437296</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
@@ -54192,23 +54192,23 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1862149954473065</t>
+          <t>1488053072699926</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
@@ -54227,23 +54227,23 @@
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>Carlos Zarb</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr"/>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Carlos Zarb</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>939653538880289</t>
+          <t>2026943771563450</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
@@ -54262,7 +54262,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -54273,12 +54273,12 @@
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1463878141656116</t>
+          <t>1003888061994637</t>
         </is>
       </c>
       <c r="F35" s="8" t="inlineStr">
@@ -54288,7 +54288,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
@@ -54297,7 +54297,7 @@
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>Rachel Williams</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
@@ -54308,12 +54308,12 @@
       <c r="C36" s="11" t="inlineStr"/>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Williams Hymie Rubetta</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>1534731544699810</t>
+          <t>2146428012843469</t>
         </is>
       </c>
       <c r="F36" s="8" t="inlineStr">
@@ -54323,7 +54323,7 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr"/>
@@ -54332,23 +54332,23 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>George Vital Zammit</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t xml:space="preserve">George Vital Zammit Kandidat PN </t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1531533181939436</t>
+          <t>864621386654273</t>
         </is>
       </c>
       <c r="F37" s="8" t="inlineStr">
@@ -54358,7 +54358,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
@@ -54367,23 +54367,23 @@
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr"/>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>1246323254060158</t>
+          <t>2423292861498917</t>
         </is>
       </c>
       <c r="F38" s="8" t="inlineStr">
@@ -54393,7 +54393,7 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr"/>
@@ -54402,7 +54402,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Julian Borg</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -54413,12 +54413,12 @@
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Julian Borg</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>26732437223117722</t>
+          <t>1690336838632544</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
@@ -54428,7 +54428,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
@@ -54437,7 +54437,7 @@
     <row r="40">
       <c r="A40" s="11" t="inlineStr">
         <is>
-          <t>Paula Mifsud Bonnici</t>
+          <t>Frank Anthony Tabone</t>
         </is>
       </c>
       <c r="B40" s="11" t="inlineStr">
@@ -54448,12 +54448,12 @@
       <c r="C40" s="11" t="inlineStr"/>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Maria Mifsud Bonnici</t>
+          <t>Frank Anthony Tabone</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
         <is>
-          <t>2435722906905478</t>
+          <t>1545046643935454</t>
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr">
@@ -54463,7 +54463,7 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr"/>
@@ -54472,23 +54472,23 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>978460398253114</t>
+          <t>1398617112285911</t>
         </is>
       </c>
       <c r="F41" s="8" t="inlineStr">
@@ -54498,7 +54498,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
@@ -54507,7 +54507,7 @@
     <row r="42">
       <c r="A42" s="11" t="inlineStr">
         <is>
-          <t>Robert Abela</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B42" s="11" t="inlineStr">
@@ -54518,12 +54518,12 @@
       <c r="C42" s="11" t="inlineStr"/>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Anthony Agius Decelis</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E42" s="11" t="inlineStr">
         <is>
-          <t>2064151104521171</t>
+          <t>1501901271598336</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
@@ -54533,7 +54533,7 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr"/>
@@ -54542,7 +54542,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Jesmond Bonello</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -54553,12 +54553,12 @@
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Bonello Jesmond</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>26918648411088542</t>
+          <t>1862149954473065</t>
         </is>
       </c>
       <c r="F43" s="8" t="inlineStr">
@@ -54568,7 +54568,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
@@ -54577,7 +54577,7 @@
     <row r="44">
       <c r="A44" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Carlos Zarb</t>
         </is>
       </c>
       <c r="B44" s="11" t="inlineStr">
@@ -54588,12 +54588,12 @@
       <c r="C44" s="11" t="inlineStr"/>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Carlos Zarb</t>
         </is>
       </c>
       <c r="E44" s="11" t="inlineStr">
         <is>
-          <t>1504143931434748</t>
+          <t>939653538880289</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
@@ -54603,7 +54603,7 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr"/>
@@ -54612,23 +54612,23 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>1518066693268355</t>
+          <t>1463878141656116</t>
         </is>
       </c>
       <c r="F45" s="8" t="inlineStr">
@@ -54647,23 +54647,23 @@
     <row r="46">
       <c r="A46" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Rachel Williams</t>
         </is>
       </c>
       <c r="B46" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr"/>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Williams Hymie Rubetta</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
         <is>
-          <t>1985551062067193</t>
+          <t>1534731544699810</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
@@ -54673,7 +54673,7 @@
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr"/>
@@ -54682,7 +54682,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Tania Borg</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -54693,12 +54693,12 @@
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Tania Borg For District 9 &amp; 10</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>974302048675707</t>
+          <t>1531533181939436</t>
         </is>
       </c>
       <c r="F47" s="8" t="inlineStr">
@@ -54708,7 +54708,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H47" t="inlineStr"/>
@@ -54717,7 +54717,7 @@
     <row r="48">
       <c r="A48" s="11" t="inlineStr">
         <is>
-          <t>Tania Borg</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B48" s="11" t="inlineStr">
@@ -54728,12 +54728,12 @@
       <c r="C48" s="11" t="inlineStr"/>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Tania Borg For District 9 &amp; 10</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
-          <t>1025067929953806</t>
+          <t>1246323254060158</t>
         </is>
       </c>
       <c r="F48" s="8" t="inlineStr">
@@ -54743,7 +54743,7 @@
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr"/>
@@ -54752,23 +54752,23 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Julian Borg</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Julian Borg</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>962084660082350</t>
+          <t>26732437223117722</t>
         </is>
       </c>
       <c r="F49" s="8" t="inlineStr">
@@ -54778,7 +54778,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H49" t="inlineStr"/>
@@ -54787,23 +54787,23 @@
     <row r="50">
       <c r="A50" s="11" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Paula Mifsud Bonnici</t>
         </is>
       </c>
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr"/>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Maria Mifsud Bonnici</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>1430222058857743</t>
+          <t>2435722906905478</t>
         </is>
       </c>
       <c r="F50" s="8" t="inlineStr">
@@ -54813,7 +54813,7 @@
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr"/>
@@ -54822,7 +54822,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>John Baptist Camilleri</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -54833,12 +54833,12 @@
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
-          <t>John Baptist Camilleri</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>993445096523240</t>
+          <t>978460398253114</t>
         </is>
       </c>
       <c r="F51" s="8" t="inlineStr">
@@ -54848,7 +54848,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
@@ -54857,23 +54857,23 @@
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
         <is>
-          <t>Julian Borg</t>
+          <t>Robert Abela</t>
         </is>
       </c>
       <c r="B52" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr"/>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Julian Borg</t>
+          <t>Anthony Agius Decelis</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
         <is>
-          <t>1006210008553971</t>
+          <t>2064151104521171</t>
         </is>
       </c>
       <c r="F52" s="8" t="inlineStr">
@@ -54883,7 +54883,7 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr"/>
@@ -54892,23 +54892,23 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Jesmond Bonello</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Bonello Jesmond</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2068362770561777</t>
+          <t>26918648411088542</t>
         </is>
       </c>
       <c r="F53" s="8" t="inlineStr">
@@ -54918,7 +54918,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H53" t="inlineStr"/>
@@ -54927,7 +54927,7 @@
     <row r="54">
       <c r="A54" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B54" s="11" t="inlineStr">
@@ -54938,12 +54938,12 @@
       <c r="C54" s="11" t="inlineStr"/>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
-          <t>996986282983288</t>
+          <t>1504143931434748</t>
         </is>
       </c>
       <c r="F54" s="8" t="inlineStr">
@@ -54953,7 +54953,7 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr"/>
@@ -54962,7 +54962,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Cressida Galea</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -54973,12 +54973,12 @@
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Cressida Galea - Ekonomista</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>4353539594976013</t>
+          <t>1518066693268355</t>
         </is>
       </c>
       <c r="F55" s="8" t="inlineStr">
@@ -54988,7 +54988,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H55" t="inlineStr"/>
@@ -54997,7 +54997,7 @@
     <row r="56">
       <c r="A56" s="11" t="inlineStr">
         <is>
-          <t>Cressida Galea</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B56" s="11" t="inlineStr">
@@ -55008,12 +55008,12 @@
       <c r="C56" s="11" t="inlineStr"/>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Cressida Galea - Ekonomista</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>1656439582071818</t>
+          <t>1985551062067193</t>
         </is>
       </c>
       <c r="F56" s="8" t="inlineStr">
@@ -55023,7 +55023,7 @@
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr"/>
@@ -55032,7 +55032,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Kaydem Schembri</t>
+          <t>Tania Borg</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -55043,12 +55043,12 @@
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Kaydem Schembri</t>
+          <t>Tania Borg For District 9 &amp; 10</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>996190969523573</t>
+          <t>974302048675707</t>
         </is>
       </c>
       <c r="F57" s="8" t="inlineStr">
@@ -55058,7 +55058,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="H57" t="inlineStr"/>
@@ -55067,23 +55067,23 @@
     <row r="58">
       <c r="A58" s="11" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Tania Borg</t>
         </is>
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
-          <t>Momentum</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr"/>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Tania Borg For District 9 &amp; 10</t>
         </is>
       </c>
       <c r="E58" s="11" t="inlineStr">
         <is>
-          <t>1625614571830540</t>
+          <t>1025067929953806</t>
         </is>
       </c>
       <c r="F58" s="8" t="inlineStr">
@@ -55093,7 +55093,7 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr"/>
@@ -55102,23 +55102,23 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>3276604689166967</t>
+          <t>962084660082350</t>
         </is>
       </c>
       <c r="F59" s="8" t="inlineStr">
@@ -55128,7 +55128,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="H59" t="inlineStr"/>
@@ -55137,7 +55137,7 @@
     <row r="60">
       <c r="A60" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="B60" s="11" t="inlineStr">
@@ -55148,12 +55148,12 @@
       <c r="C60" s="11" t="inlineStr"/>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="E60" s="11" t="inlineStr">
         <is>
-          <t>2115618699296224</t>
+          <t>1430222058857743</t>
         </is>
       </c>
       <c r="F60" s="8" t="inlineStr">
@@ -55163,7 +55163,7 @@
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr"/>
@@ -55172,23 +55172,23 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>John Baptist Camilleri</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>John Baptist Camilleri</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>949145677752982</t>
+          <t>993445096523240</t>
         </is>
       </c>
       <c r="F61" s="8" t="inlineStr">
@@ -55198,7 +55198,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H61" t="inlineStr"/>
@@ -55207,23 +55207,23 @@
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Julian Borg</t>
         </is>
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>Momentum</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr"/>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Julian Borg</t>
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr">
         <is>
-          <t>1470892497314849</t>
+          <t>1006210008553971</t>
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
@@ -55233,7 +55233,7 @@
       </c>
       <c r="G62" s="11" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H62" s="11" t="inlineStr"/>
@@ -55242,23 +55242,23 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Momentum</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>1997023797841290</t>
+          <t>2068362770561777</t>
         </is>
       </c>
       <c r="F63" s="8" t="inlineStr">
@@ -55268,7 +55268,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H63" t="inlineStr"/>
@@ -55277,7 +55277,7 @@
     <row r="64">
       <c r="A64" s="11" t="inlineStr">
         <is>
-          <t>Lorna Borg Vassallo</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B64" s="11" t="inlineStr">
@@ -55288,12 +55288,12 @@
       <c r="C64" s="11" t="inlineStr"/>
       <c r="D64" s="11" t="inlineStr">
         <is>
-          <t>Lorna Borġ Vassallo</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E64" s="11" t="inlineStr">
         <is>
-          <t>982543764707676</t>
+          <t>996986282983288</t>
         </is>
       </c>
       <c r="F64" s="8" t="inlineStr">
@@ -55303,7 +55303,7 @@
       </c>
       <c r="G64" s="11" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H64" s="11" t="inlineStr"/>
@@ -55312,23 +55312,23 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>John Baptist Camilleri</t>
+          <t>Cressida Galea</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
-          <t>John Baptist Camilleri</t>
+          <t>Cressida Galea - Ekonomista</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>35349534414693500</t>
+          <t>4353539594976013</t>
         </is>
       </c>
       <c r="F65" s="8" t="inlineStr">
@@ -55338,7 +55338,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H65" t="inlineStr"/>
@@ -55347,7 +55347,7 @@
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
         <is>
-          <t>Katya De Giovanni</t>
+          <t>Cressida Galea</t>
         </is>
       </c>
       <c r="B66" s="11" t="inlineStr">
@@ -55358,12 +55358,12 @@
       <c r="C66" s="11" t="inlineStr"/>
       <c r="D66" s="11" t="inlineStr">
         <is>
-          <t>Katya De Giovanni</t>
+          <t>Cressida Galea - Ekonomista</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
         <is>
-          <t>26625959597085054</t>
+          <t>1656439582071818</t>
         </is>
       </c>
       <c r="F66" s="8" t="inlineStr">
@@ -55373,7 +55373,7 @@
       </c>
       <c r="G66" s="11" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H66" s="11" t="inlineStr"/>
@@ -55382,23 +55382,23 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Kaydem Schembri</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Kaydem Schembri</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>909198525476235</t>
+          <t>996190969523573</t>
         </is>
       </c>
       <c r="F67" s="8" t="inlineStr">
@@ -55408,7 +55408,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H67" t="inlineStr"/>
@@ -55417,23 +55417,23 @@
     <row r="68">
       <c r="A68" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="B68" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C68" s="11" t="inlineStr"/>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
         <is>
-          <t>2050566099220285</t>
+          <t>1625614571830540</t>
         </is>
       </c>
       <c r="F68" s="8" t="inlineStr">
@@ -55443,7 +55443,7 @@
       </c>
       <c r="G68" s="11" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H68" s="11" t="inlineStr"/>
@@ -55452,7 +55452,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -55463,12 +55463,12 @@
       <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>1677247313280464</t>
+          <t>3276604689166967</t>
         </is>
       </c>
       <c r="F69" s="8" t="inlineStr">
@@ -55478,7 +55478,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H69" t="inlineStr"/>
@@ -55487,7 +55487,7 @@
     <row r="70">
       <c r="A70" s="11" t="inlineStr">
         <is>
-          <t>Nigel Vella</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B70" s="11" t="inlineStr">
@@ -55498,12 +55498,12 @@
       <c r="C70" s="11" t="inlineStr"/>
       <c r="D70" s="11" t="inlineStr">
         <is>
-          <t>Nigel Vella</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
         <is>
-          <t>1478044677100859</t>
+          <t>2115618699296224</t>
         </is>
       </c>
       <c r="F70" s="8" t="inlineStr">
@@ -55513,7 +55513,7 @@
       </c>
       <c r="G70" s="11" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H70" s="11" t="inlineStr"/>
@@ -55522,7 +55522,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Lorna Borg Vassallo</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -55533,12 +55533,12 @@
       <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Lorna Borġ Vassallo</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>942778361908557</t>
+          <t>949145677752982</t>
         </is>
       </c>
       <c r="F71" s="8" t="inlineStr">
@@ -55548,7 +55548,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H71" t="inlineStr"/>
@@ -55557,23 +55557,23 @@
     <row r="72">
       <c r="A72" s="11" t="inlineStr">
         <is>
-          <t>Lorna Borg Vassallo</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="B72" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C72" s="11" t="inlineStr"/>
       <c r="D72" s="11" t="inlineStr">
         <is>
-          <t>Lorna Borġ Vassallo</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
         <is>
-          <t>984647040762034</t>
+          <t>1470892497314849</t>
         </is>
       </c>
       <c r="F72" s="8" t="inlineStr">
@@ -55583,11 +55583,291 @@
       </c>
       <c r="G72" s="11" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H72" s="11" t="inlineStr"/>
       <c r="I72" s="11" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Matthew Agius</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Momentum</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Matthew Agius</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>1997023797841290</t>
+        </is>
+      </c>
+      <c r="F73" s="8" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="11" t="inlineStr">
+        <is>
+          <t>Lorna Borg Vassallo</t>
+        </is>
+      </c>
+      <c r="B74" s="11" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C74" s="11" t="inlineStr"/>
+      <c r="D74" s="11" t="inlineStr">
+        <is>
+          <t>Lorna Borġ Vassallo</t>
+        </is>
+      </c>
+      <c r="E74" s="11" t="inlineStr">
+        <is>
+          <t>982543764707676</t>
+        </is>
+      </c>
+      <c r="F74" s="8" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="G74" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="H74" s="11" t="inlineStr"/>
+      <c r="I74" s="11" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>John Baptist Camilleri</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>PN</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>John Baptist Camilleri</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>35349534414693500</t>
+        </is>
+      </c>
+      <c r="F75" s="8" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="inlineStr">
+        <is>
+          <t>Katya De Giovanni</t>
+        </is>
+      </c>
+      <c r="B76" s="11" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C76" s="11" t="inlineStr"/>
+      <c r="D76" s="11" t="inlineStr">
+        <is>
+          <t>Katya De Giovanni</t>
+        </is>
+      </c>
+      <c r="E76" s="11" t="inlineStr">
+        <is>
+          <t>26625959597085054</t>
+        </is>
+      </c>
+      <c r="F76" s="8" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="G76" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="H76" s="11" t="inlineStr"/>
+      <c r="I76" s="11" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Edward Cassar Delia</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Edward Cassar Delia</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>2050566099220285</t>
+        </is>
+      </c>
+      <c r="F77" s="8" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="11" t="inlineStr">
+        <is>
+          <t>Nigel Vella</t>
+        </is>
+      </c>
+      <c r="B78" s="11" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C78" s="11" t="inlineStr"/>
+      <c r="D78" s="11" t="inlineStr">
+        <is>
+          <t>Nigel Vella</t>
+        </is>
+      </c>
+      <c r="E78" s="11" t="inlineStr">
+        <is>
+          <t>1478044677100859</t>
+        </is>
+      </c>
+      <c r="F78" s="8" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="G78" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="H78" s="11" t="inlineStr"/>
+      <c r="I78" s="11" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Lorna Borg Vassallo</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Lorna Borġ Vassallo</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>942778361908557</t>
+        </is>
+      </c>
+      <c r="F79" s="8" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="inlineStr">
+        <is>
+          <t>Lorna Borg Vassallo</t>
+        </is>
+      </c>
+      <c r="B80" s="11" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C80" s="11" t="inlineStr"/>
+      <c r="D80" s="11" t="inlineStr">
+        <is>
+          <t>Lorna Borġ Vassallo</t>
+        </is>
+      </c>
+      <c r="E80" s="11" t="inlineStr">
+        <is>
+          <t>984647040762034</t>
+        </is>
+      </c>
+      <c r="F80" s="8" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="G80" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="H80" s="11" t="inlineStr"/>
+      <c r="I80" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -55660,6 +55940,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F79" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F80" r:id="rId77"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto(MT): 3h refresh 2026-05-17T11:38Z
</commit_message>
<xml_diff>
--- a/summary_2026-05-17.xlsx
+++ b/summary_2026-05-17.xlsx
@@ -575,10 +575,10 @@
         <v>332</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>403</v>
+        <v>432</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>744</v>
+        <v>773</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>447912</v>
@@ -765,20 +765,20 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΒΟΛΤ</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>0</v>
@@ -790,59 +790,55 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ΒΟΛΤ</t>
+          <t>ΔΕΚ</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D13" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E13" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>8997</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>297</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>ΔΕΚ</t>
+          <t>ΔΑ</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>8997</v>
+        <v>0</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>297</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>ΔΑ</t>
-        </is>
-      </c>
+      <c r="A15" t="inlineStr"/>
       <c r="B15" t="n">
         <v>0</v>
       </c>
@@ -850,10 +846,10 @@
         <v>11</v>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E15" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
@@ -863,18 +859,22 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr"/>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>ΕΝΕΡΓΟΙ ΠΟΛΙΤΕΣ</t>
+        </is>
+      </c>
       <c r="B16" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>0</v>
@@ -886,17 +886,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ΕΝΕΡΓΟΙ ΠΟΛΙΤΕΣ</t>
+          <t>ΕΔΕΚ</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D17" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E17" t="n">
         <v>13</v>
@@ -32067,7 +32067,7 @@
       </c>
       <c r="B532" s="3" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C532" s="3" t="inlineStr">
@@ -32119,7 +32119,7 @@
       </c>
       <c r="B533" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C533" t="inlineStr">
@@ -32171,7 +32171,7 @@
       </c>
       <c r="B534" s="3" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C534" s="3" t="inlineStr">
@@ -32223,7 +32223,7 @@
       </c>
       <c r="B535" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C535" t="inlineStr">
@@ -32275,7 +32275,7 @@
       </c>
       <c r="B536" s="3" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C536" s="3" t="inlineStr">
@@ -32327,7 +32327,7 @@
       </c>
       <c r="B537" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C537" t="inlineStr">
@@ -32379,7 +32379,7 @@
       </c>
       <c r="B538" s="3" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C538" s="3" t="inlineStr">
@@ -32431,7 +32431,7 @@
       </c>
       <c r="B539" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C539" t="inlineStr">
@@ -32483,7 +32483,7 @@
       </c>
       <c r="B540" s="3" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C540" s="3" t="inlineStr">
@@ -32535,7 +32535,7 @@
       </c>
       <c r="B541" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C541" t="inlineStr">
@@ -32587,7 +32587,7 @@
       </c>
       <c r="B542" s="3" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C542" s="3" t="inlineStr">
@@ -32639,7 +32639,7 @@
       </c>
       <c r="B543" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C543" t="inlineStr">
@@ -32691,7 +32691,7 @@
       </c>
       <c r="B544" s="3" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C544" s="3" t="inlineStr">
@@ -32743,7 +32743,7 @@
       </c>
       <c r="B545" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C545" t="inlineStr">
@@ -32795,7 +32795,7 @@
       </c>
       <c r="B546" s="3" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C546" s="3" t="inlineStr">
@@ -32847,7 +32847,7 @@
       </c>
       <c r="B547" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C547" t="inlineStr">
@@ -32899,7 +32899,7 @@
       </c>
       <c r="B548" s="3" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C548" s="3" t="inlineStr">
@@ -32951,7 +32951,7 @@
       </c>
       <c r="B549" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C549" t="inlineStr">
@@ -33003,7 +33003,7 @@
       </c>
       <c r="B550" s="3" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C550" s="3" t="inlineStr">
@@ -33055,7 +33055,7 @@
       </c>
       <c r="B551" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C551" t="inlineStr">
@@ -33107,7 +33107,7 @@
       </c>
       <c r="B552" s="3" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C552" s="3" t="inlineStr">
@@ -33159,7 +33159,7 @@
       </c>
       <c r="B553" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C553" t="inlineStr">
@@ -33211,7 +33211,7 @@
       </c>
       <c r="B554" s="3" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C554" s="3" t="inlineStr">
@@ -33263,7 +33263,7 @@
       </c>
       <c r="B555" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C555" t="inlineStr">
@@ -33315,7 +33315,7 @@
       </c>
       <c r="B556" s="3" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C556" s="3" t="inlineStr">
@@ -33367,7 +33367,7 @@
       </c>
       <c r="B557" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C557" t="inlineStr">
@@ -33419,7 +33419,7 @@
       </c>
       <c r="B558" s="3" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C558" s="3" t="inlineStr">
@@ -40339,7 +40339,7 @@
       </c>
       <c r="B692" s="3" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C692" s="3" t="inlineStr">
@@ -40391,7 +40391,7 @@
       </c>
       <c r="B693" t="inlineStr">
         <is>
-          <t>ΕΔΕΚ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C693" t="inlineStr">

</xml_diff>

<commit_message>
auto(MT): 3h refresh 2026-05-17T14:34Z
</commit_message>
<xml_diff>
--- a/summary_2026-05-17.xlsx
+++ b/summary_2026-05-17.xlsx
@@ -53106,10 +53106,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C5" t="n">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="D5" t="n">
         <v>58</v>
@@ -53156,10 +53156,10 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1358</v>
+        <v>1355</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>125</v>
@@ -53185,7 +53185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I80"/>
+  <dimension ref="A1:I83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -53607,23 +53607,23 @@
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr"/>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>1680974129907056</t>
+          <t>4401025156884497</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -53658,7 +53658,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1479722413058169</t>
+          <t>1680974129907056</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -53677,7 +53677,7 @@
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
@@ -53688,12 +53688,12 @@
       <c r="C16" s="11" t="inlineStr"/>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>1426917766136513</t>
+          <t>1479722413058169</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -53712,7 +53712,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Vania Agius Tabone</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -53723,12 +53723,12 @@
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Vania Agius Tabone</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1321288733281834</t>
+          <t>1426917766136513</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -53747,23 +53747,23 @@
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Vania Agius Tabone</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr"/>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Vania Agius Tabone</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>2380595315785369</t>
+          <t>1321288733281834</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -53798,7 +53798,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1683215979770872</t>
+          <t>2380595315785369</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -53817,23 +53817,23 @@
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr"/>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>3871030129694577</t>
+          <t>1683215979770872</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -53852,23 +53852,23 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>945783808284948</t>
+          <t>1644456073494625</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -53887,7 +53887,7 @@
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
@@ -53898,12 +53898,12 @@
       <c r="C22" s="11" t="inlineStr"/>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>1350786307104546</t>
+          <t>3871030129694577</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -53922,7 +53922,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -53933,12 +53933,12 @@
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>873330299113401</t>
+          <t>945783808284948</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -53973,7 +53973,7 @@
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>1294864578834169</t>
+          <t>1350786307104546</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -53992,7 +53992,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Miriam Dalli</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -54003,12 +54003,12 @@
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Malta ESG Alliance</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2377088586134238</t>
+          <t>873330299113401</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
@@ -54027,7 +54027,7 @@
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>Samantha Pace Gasan</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
@@ -54038,12 +54038,12 @@
       <c r="C26" s="11" t="inlineStr"/>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Samantha Pace Gasan</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>983555364558689</t>
+          <t>1294864578834169</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -54062,7 +54062,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Miriam Dalli</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -54073,12 +54073,12 @@
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Malta ESG Alliance</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1272070931325786</t>
+          <t>2377088586134238</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
@@ -54097,7 +54097,7 @@
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Samantha Pace Gasan</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
@@ -54108,12 +54108,12 @@
       <c r="C28" s="11" t="inlineStr"/>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Samantha Pace Gasan</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>2431998763969509</t>
+          <t>983555364558689</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
@@ -54132,7 +54132,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>James Grech</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -54143,12 +54143,12 @@
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>James Grech</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>971268672293806</t>
+          <t>1272070931325786</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
@@ -54167,7 +54167,7 @@
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>James Grech</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
@@ -54178,12 +54178,12 @@
       <c r="C30" s="11" t="inlineStr"/>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>James Grech</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>991693409986643</t>
+          <t>2431998763969509</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
@@ -54218,7 +54218,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2662232900814818</t>
+          <t>971268672293806</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
@@ -54237,23 +54237,23 @@
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>Alex Borg</t>
+          <t>James Grech</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr"/>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>James Grech</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>958905883437296</t>
+          <t>991693409986643</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
@@ -54263,7 +54263,7 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr"/>
@@ -54272,23 +54272,23 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>James Grech</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>James Grech</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1488053072699926</t>
+          <t>2662232900814818</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
@@ -54298,7 +54298,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
@@ -54307,7 +54307,7 @@
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Alex Borg</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
@@ -54318,12 +54318,12 @@
       <c r="C34" s="11" t="inlineStr"/>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>2026943771563450</t>
+          <t>958905883437296</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
@@ -54342,7 +54342,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -54353,12 +54353,12 @@
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1003888061994637</t>
+          <t>1488053072699926</t>
         </is>
       </c>
       <c r="F35" s="8" t="inlineStr">
@@ -54377,7 +54377,7 @@
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
@@ -54388,12 +54388,12 @@
       <c r="C36" s="11" t="inlineStr"/>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>2146428012843469</t>
+          <t>2026943771563450</t>
         </is>
       </c>
       <c r="F36" s="8" t="inlineStr">
@@ -54412,7 +54412,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>George Vital Zammit</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -54423,12 +54423,12 @@
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">George Vital Zammit Kandidat PN </t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>864621386654273</t>
+          <t>1003888061994637</t>
         </is>
       </c>
       <c r="F37" s="8" t="inlineStr">
@@ -54447,7 +54447,7 @@
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
@@ -54458,12 +54458,12 @@
       <c r="C38" s="11" t="inlineStr"/>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>2423292861498917</t>
+          <t>2146428012843469</t>
         </is>
       </c>
       <c r="F38" s="8" t="inlineStr">
@@ -54482,7 +54482,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>George Vital Zammit</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -54493,12 +54493,12 @@
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t xml:space="preserve">George Vital Zammit Kandidat PN </t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1690336838632544</t>
+          <t>864621386654273</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
@@ -54517,7 +54517,7 @@
     <row r="40">
       <c r="A40" s="11" t="inlineStr">
         <is>
-          <t>Frank Anthony Tabone</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="B40" s="11" t="inlineStr">
@@ -54528,12 +54528,12 @@
       <c r="C40" s="11" t="inlineStr"/>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Frank Anthony Tabone</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
         <is>
-          <t>1545046643935454</t>
+          <t>2423292861498917</t>
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr">
@@ -54552,23 +54552,23 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1398617112285911</t>
+          <t>1690336838632544</t>
         </is>
       </c>
       <c r="F41" s="8" t="inlineStr">
@@ -54587,23 +54587,23 @@
     <row r="42">
       <c r="A42" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Frank Anthony Tabone</t>
         </is>
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr"/>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Frank Anthony Tabone</t>
         </is>
       </c>
       <c r="E42" s="11" t="inlineStr">
         <is>
-          <t>1501901271598336</t>
+          <t>1545046643935454</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
@@ -54622,7 +54622,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -54633,12 +54633,12 @@
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1862149954473065</t>
+          <t>1398617112285911</t>
         </is>
       </c>
       <c r="F43" s="8" t="inlineStr">
@@ -54657,7 +54657,7 @@
     <row r="44">
       <c r="A44" s="11" t="inlineStr">
         <is>
-          <t>Carlos Zarb</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B44" s="11" t="inlineStr">
@@ -54668,12 +54668,12 @@
       <c r="C44" s="11" t="inlineStr"/>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Carlos Zarb</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E44" s="11" t="inlineStr">
         <is>
-          <t>939653538880289</t>
+          <t>1501901271598336</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
@@ -54692,23 +54692,23 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>1463878141656116</t>
+          <t>1862149954473065</t>
         </is>
       </c>
       <c r="F45" s="8" t="inlineStr">
@@ -54718,7 +54718,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="H45" t="inlineStr"/>
@@ -54727,23 +54727,23 @@
     <row r="46">
       <c r="A46" s="11" t="inlineStr">
         <is>
-          <t>Rachel Williams</t>
+          <t>Carlos Zarb</t>
         </is>
       </c>
       <c r="B46" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr"/>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Williams Hymie Rubetta</t>
+          <t>Carlos Zarb</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
         <is>
-          <t>1534731544699810</t>
+          <t>939653538880289</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
@@ -54753,7 +54753,7 @@
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr"/>
@@ -54762,23 +54762,23 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>1531533181939436</t>
+          <t>1463878141656116</t>
         </is>
       </c>
       <c r="F47" s="8" t="inlineStr">
@@ -54797,23 +54797,23 @@
     <row r="48">
       <c r="A48" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Rachel Williams</t>
         </is>
       </c>
       <c r="B48" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr"/>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Williams Hymie Rubetta</t>
         </is>
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
-          <t>1246323254060158</t>
+          <t>1534731544699810</t>
         </is>
       </c>
       <c r="F48" s="8" t="inlineStr">
@@ -54832,23 +54832,23 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Julian Borg</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Julian Borg</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>26732437223117722</t>
+          <t>1531533181939436</t>
         </is>
       </c>
       <c r="F49" s="8" t="inlineStr">
@@ -54867,23 +54867,23 @@
     <row r="50">
       <c r="A50" s="11" t="inlineStr">
         <is>
-          <t>Paula Mifsud Bonnici</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr"/>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Maria Mifsud Bonnici</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>2435722906905478</t>
+          <t>1246323254060158</t>
         </is>
       </c>
       <c r="F50" s="8" t="inlineStr">
@@ -54902,7 +54902,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Julian Borg</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -54913,12 +54913,12 @@
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Julian Borg</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>978460398253114</t>
+          <t>26732437223117722</t>
         </is>
       </c>
       <c r="F51" s="8" t="inlineStr">
@@ -54937,23 +54937,23 @@
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
         <is>
-          <t>Robert Abela</t>
+          <t>Paula Mifsud Bonnici</t>
         </is>
       </c>
       <c r="B52" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr"/>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Anthony Agius Decelis</t>
+          <t>Maria Mifsud Bonnici</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
         <is>
-          <t>2064151104521171</t>
+          <t>2435722906905478</t>
         </is>
       </c>
       <c r="F52" s="8" t="inlineStr">
@@ -54972,23 +54972,23 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Jesmond Bonello</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Bonello Jesmond</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>26918648411088542</t>
+          <t>978460398253114</t>
         </is>
       </c>
       <c r="F53" s="8" t="inlineStr">
@@ -55007,7 +55007,7 @@
     <row r="54">
       <c r="A54" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Robert Abela</t>
         </is>
       </c>
       <c r="B54" s="11" t="inlineStr">
@@ -55018,12 +55018,12 @@
       <c r="C54" s="11" t="inlineStr"/>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Anthony Agius Decelis</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
-          <t>1504143931434748</t>
+          <t>2064151104521171</t>
         </is>
       </c>
       <c r="F54" s="8" t="inlineStr">
@@ -55042,7 +55042,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Jesmond Bonello</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -55053,12 +55053,12 @@
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Bonello Jesmond</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>1518066693268355</t>
+          <t>26918648411088542</t>
         </is>
       </c>
       <c r="F55" s="8" t="inlineStr">
@@ -55077,7 +55077,7 @@
     <row r="56">
       <c r="A56" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B56" s="11" t="inlineStr">
@@ -55088,12 +55088,12 @@
       <c r="C56" s="11" t="inlineStr"/>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>1985551062067193</t>
+          <t>1504143931434748</t>
         </is>
       </c>
       <c r="F56" s="8" t="inlineStr">
@@ -55103,7 +55103,7 @@
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr"/>
@@ -55112,7 +55112,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Tania Borg</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -55123,12 +55123,12 @@
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Tania Borg For District 9 &amp; 10</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>974302048675707</t>
+          <t>1518066693268355</t>
         </is>
       </c>
       <c r="F57" s="8" t="inlineStr">
@@ -55138,7 +55138,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H57" t="inlineStr"/>
@@ -55147,7 +55147,7 @@
     <row r="58">
       <c r="A58" s="11" t="inlineStr">
         <is>
-          <t>Tania Borg</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B58" s="11" t="inlineStr">
@@ -55158,12 +55158,12 @@
       <c r="C58" s="11" t="inlineStr"/>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Tania Borg For District 9 &amp; 10</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E58" s="11" t="inlineStr">
         <is>
-          <t>1025067929953806</t>
+          <t>1985551062067193</t>
         </is>
       </c>
       <c r="F58" s="8" t="inlineStr">
@@ -55182,7 +55182,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Tania Borg</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -55193,12 +55193,12 @@
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Tania Borg For District 9 &amp; 10</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>962084660082350</t>
+          <t>974302048675707</t>
         </is>
       </c>
       <c r="F59" s="8" t="inlineStr">
@@ -55217,7 +55217,7 @@
     <row r="60">
       <c r="A60" s="11" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Tania Borg</t>
         </is>
       </c>
       <c r="B60" s="11" t="inlineStr">
@@ -55228,12 +55228,12 @@
       <c r="C60" s="11" t="inlineStr"/>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Tania Borg For District 9 &amp; 10</t>
         </is>
       </c>
       <c r="E60" s="11" t="inlineStr">
         <is>
-          <t>1430222058857743</t>
+          <t>1025067929953806</t>
         </is>
       </c>
       <c r="F60" s="8" t="inlineStr">
@@ -55252,23 +55252,23 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>John Baptist Camilleri</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
-          <t>John Baptist Camilleri</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>993445096523240</t>
+          <t>962084660082350</t>
         </is>
       </c>
       <c r="F61" s="8" t="inlineStr">
@@ -55278,7 +55278,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="H61" t="inlineStr"/>
@@ -55287,23 +55287,23 @@
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
         <is>
-          <t>Julian Borg</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr"/>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>Julian Borg</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr">
         <is>
-          <t>1006210008553971</t>
+          <t>1430222058857743</t>
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
@@ -55313,7 +55313,7 @@
       </c>
       <c r="G62" s="11" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="H62" s="11" t="inlineStr"/>
@@ -55322,7 +55322,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>John Baptist Camilleri</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -55333,12 +55333,12 @@
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>John Baptist Camilleri</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>2068362770561777</t>
+          <t>993445096523240</t>
         </is>
       </c>
       <c r="F63" s="8" t="inlineStr">
@@ -55357,23 +55357,23 @@
     <row r="64">
       <c r="A64" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Julian Borg</t>
         </is>
       </c>
       <c r="B64" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C64" s="11" t="inlineStr"/>
       <c r="D64" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Julian Borg</t>
         </is>
       </c>
       <c r="E64" s="11" t="inlineStr">
         <is>
-          <t>996986282983288</t>
+          <t>1006210008553971</t>
         </is>
       </c>
       <c r="F64" s="8" t="inlineStr">
@@ -55392,23 +55392,23 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Cressida Galea</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Cressida Galea - Ekonomista</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>4353539594976013</t>
+          <t>2068362770561777</t>
         </is>
       </c>
       <c r="F65" s="8" t="inlineStr">
@@ -55427,7 +55427,7 @@
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
         <is>
-          <t>Cressida Galea</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B66" s="11" t="inlineStr">
@@ -55438,12 +55438,12 @@
       <c r="C66" s="11" t="inlineStr"/>
       <c r="D66" s="11" t="inlineStr">
         <is>
-          <t>Cressida Galea - Ekonomista</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
         <is>
-          <t>1656439582071818</t>
+          <t>996986282983288</t>
         </is>
       </c>
       <c r="F66" s="8" t="inlineStr">
@@ -55462,7 +55462,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Kaydem Schembri</t>
+          <t>Cressida Galea</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -55473,12 +55473,12 @@
       <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Kaydem Schembri</t>
+          <t>Cressida Galea - Ekonomista</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>996190969523573</t>
+          <t>4353539594976013</t>
         </is>
       </c>
       <c r="F67" s="8" t="inlineStr">
@@ -55497,23 +55497,23 @@
     <row r="68">
       <c r="A68" s="11" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Cressida Galea</t>
         </is>
       </c>
       <c r="B68" s="11" t="inlineStr">
         <is>
-          <t>Momentum</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C68" s="11" t="inlineStr"/>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Cressida Galea - Ekonomista</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
         <is>
-          <t>1625614571830540</t>
+          <t>1656439582071818</t>
         </is>
       </c>
       <c r="F68" s="8" t="inlineStr">
@@ -55532,23 +55532,23 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>Kaydem Schembri</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>Kaydem Schembri</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>3276604689166967</t>
+          <t>996190969523573</t>
         </is>
       </c>
       <c r="F69" s="8" t="inlineStr">
@@ -55558,7 +55558,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H69" t="inlineStr"/>
@@ -55567,23 +55567,23 @@
     <row r="70">
       <c r="A70" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="B70" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C70" s="11" t="inlineStr"/>
       <c r="D70" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
         <is>
-          <t>2115618699296224</t>
+          <t>1625614571830540</t>
         </is>
       </c>
       <c r="F70" s="8" t="inlineStr">
@@ -55593,7 +55593,7 @@
       </c>
       <c r="G70" s="11" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H70" s="11" t="inlineStr"/>
@@ -55602,23 +55602,23 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>949145677752982</t>
+          <t>3276604689166967</t>
         </is>
       </c>
       <c r="F71" s="8" t="inlineStr">
@@ -55637,23 +55637,23 @@
     <row r="72">
       <c r="A72" s="11" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B72" s="11" t="inlineStr">
         <is>
-          <t>Momentum</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C72" s="11" t="inlineStr"/>
       <c r="D72" s="11" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
         <is>
-          <t>1470892497314849</t>
+          <t>2115618699296224</t>
         </is>
       </c>
       <c r="F72" s="8" t="inlineStr">
@@ -55672,23 +55672,23 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Momentum</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>1997023797841290</t>
+          <t>949145677752982</t>
         </is>
       </c>
       <c r="F73" s="8" t="inlineStr">
@@ -55707,23 +55707,23 @@
     <row r="74">
       <c r="A74" s="11" t="inlineStr">
         <is>
-          <t>Lorna Borg Vassallo</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="B74" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C74" s="11" t="inlineStr"/>
       <c r="D74" s="11" t="inlineStr">
         <is>
-          <t>Lorna Borġ Vassallo</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
         <is>
-          <t>982543764707676</t>
+          <t>1470892497314849</t>
         </is>
       </c>
       <c r="F74" s="8" t="inlineStr">
@@ -55742,23 +55742,23 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>John Baptist Camilleri</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr">
         <is>
-          <t>John Baptist Camilleri</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>35349534414693500</t>
+          <t>1997023797841290</t>
         </is>
       </c>
       <c r="F75" s="8" t="inlineStr">
@@ -55768,7 +55768,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H75" t="inlineStr"/>
@@ -55777,7 +55777,7 @@
     <row r="76">
       <c r="A76" s="11" t="inlineStr">
         <is>
-          <t>Katya De Giovanni</t>
+          <t>Lorna Borg Vassallo</t>
         </is>
       </c>
       <c r="B76" s="11" t="inlineStr">
@@ -55788,12 +55788,12 @@
       <c r="C76" s="11" t="inlineStr"/>
       <c r="D76" s="11" t="inlineStr">
         <is>
-          <t>Katya De Giovanni</t>
+          <t>Lorna Borġ Vassallo</t>
         </is>
       </c>
       <c r="E76" s="11" t="inlineStr">
         <is>
-          <t>26625959597085054</t>
+          <t>982543764707676</t>
         </is>
       </c>
       <c r="F76" s="8" t="inlineStr">
@@ -55803,7 +55803,7 @@
       </c>
       <c r="G76" s="11" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H76" s="11" t="inlineStr"/>
@@ -55812,23 +55812,23 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>John Baptist Camilleri</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>John Baptist Camilleri</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>2050566099220285</t>
+          <t>35349534414693500</t>
         </is>
       </c>
       <c r="F77" s="8" t="inlineStr">
@@ -55838,7 +55838,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H77" t="inlineStr"/>
@@ -55847,7 +55847,7 @@
     <row r="78">
       <c r="A78" s="11" t="inlineStr">
         <is>
-          <t>Nigel Vella</t>
+          <t>Katya De Giovanni</t>
         </is>
       </c>
       <c r="B78" s="11" t="inlineStr">
@@ -55858,12 +55858,12 @@
       <c r="C78" s="11" t="inlineStr"/>
       <c r="D78" s="11" t="inlineStr">
         <is>
-          <t>Nigel Vella</t>
+          <t>Katya De Giovanni</t>
         </is>
       </c>
       <c r="E78" s="11" t="inlineStr">
         <is>
-          <t>1478044677100859</t>
+          <t>26625959597085054</t>
         </is>
       </c>
       <c r="F78" s="8" t="inlineStr">
@@ -55873,7 +55873,7 @@
       </c>
       <c r="G78" s="11" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="H78" s="11" t="inlineStr"/>
@@ -55882,23 +55882,23 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Lorna Borg Vassallo</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C79" t="inlineStr"/>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Lorna Borġ Vassallo</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>942778361908557</t>
+          <t>909198525476235</t>
         </is>
       </c>
       <c r="F79" s="8" t="inlineStr">
@@ -55908,7 +55908,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="H79" t="inlineStr"/>
@@ -55917,7 +55917,7 @@
     <row r="80">
       <c r="A80" s="11" t="inlineStr">
         <is>
-          <t>Lorna Borg Vassallo</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B80" s="11" t="inlineStr">
@@ -55928,12 +55928,12 @@
       <c r="C80" s="11" t="inlineStr"/>
       <c r="D80" s="11" t="inlineStr">
         <is>
-          <t>Lorna Borġ Vassallo</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E80" s="11" t="inlineStr">
         <is>
-          <t>984647040762034</t>
+          <t>2050566099220285</t>
         </is>
       </c>
       <c r="F80" s="8" t="inlineStr">
@@ -55943,11 +55943,116 @@
       </c>
       <c r="G80" s="11" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="H80" s="11" t="inlineStr"/>
       <c r="I80" s="11" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Nigel Vella</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Nigel Vella</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>1478044677100859</t>
+        </is>
+      </c>
+      <c r="F81" s="8" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="inlineStr">
+        <is>
+          <t>Lorna Borg Vassallo</t>
+        </is>
+      </c>
+      <c r="B82" s="11" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C82" s="11" t="inlineStr"/>
+      <c r="D82" s="11" t="inlineStr">
+        <is>
+          <t>Lorna Borġ Vassallo</t>
+        </is>
+      </c>
+      <c r="E82" s="11" t="inlineStr">
+        <is>
+          <t>942778361908557</t>
+        </is>
+      </c>
+      <c r="F82" s="8" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="G82" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="H82" s="11" t="inlineStr"/>
+      <c r="I82" s="11" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Lorna Borg Vassallo</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr"/>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Lorna Borġ Vassallo</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>984647040762034</t>
+        </is>
+      </c>
+      <c r="F83" s="8" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -56028,6 +56133,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F79" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F80" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F81" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F82" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F83" r:id="rId80"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>